<commit_message>
fix: Correção de bugs no ImportarPlanilha
</commit_message>
<xml_diff>
--- a/BibliotecaRHC.Web/public/assets/modelo-importacao.xlsx
+++ b/BibliotecaRHC.Web/public/assets/modelo-importacao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/26f98e05a58fbc4a/Documentos/Livros/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D2B2542E-8A35-46C6-B36A-1BA7AD50782D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8D9E35B3-3CD0-4582-B400-2ECC29C569BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Nº</t>
   </si>
@@ -63,6 +63,12 @@
   </si>
   <si>
     <t>Aquisição</t>
+  </si>
+  <si>
+    <t>Lido</t>
+  </si>
+  <si>
+    <t>AnoUltimaLeitura</t>
   </si>
 </sst>
 </file>
@@ -537,6 +543,8 @@
     <col min="7" max="7" width="32.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="33.7109375" customWidth="1"/>
     <col min="9" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" customWidth="1"/>
+    <col min="11" max="11" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="18.75">
@@ -567,8 +575,12 @@
       <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>10</v>
+      </c>
       <c r="L1" s="3"/>
       <c r="M1" s="3"/>
       <c r="N1" s="3"/>

</xml_diff>